<commit_message>
Evidence nese stav žádosti o doplnění
Sešit dodavatele v objednavky.xlsx měl poslední sloupec Kompletní, takže
u neúplné faktury bylo vidět, že něco chybí, ale ne že se o doplnění už
psalo — to leželo jen v kontrola-<datum>.xlsx toho dne. Přibývá sloupec
Žádost odeslána: čas odeslání, nebo „připraveno, čeká na konektor".

Skill zapisuje čas na tři místa (sešit dodavatele, Přehled, evidence) a
nově drží text v sešitu a text, který odejde, slovo od slova stejný.
Runbook dostal řádek o faktuře, která je v evidenci dvakrát, protože její
PDF mezitím ze vstup/ zmizelo.

Lekce: zadání naplánované úlohy srovnané se skillem, strom projektu a
poznámka o konektoru zmiňují nový sloupec. Zip přebalen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cviceni/faktury-kontrola/data/objednavky.xlsx
+++ b/cviceni/faktury-kontrola/data/objednavky.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stavebniny Morava" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nářadí Profi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elektro Dvořák" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VTS Technik" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Barvy Piekarová" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Stavebniny Morava" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Nářadí Profi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Elektro Dvořák" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="VTS Technik" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Barvy Piekarová" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,6 +481,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Kompletní</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Žádost odeslána</t>
         </is>
       </c>
     </row>
@@ -534,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -545,6 +551,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -586,6 +593,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Kompletní</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Žádost odeslána</t>
         </is>
       </c>
     </row>
@@ -640,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -651,6 +663,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -694,6 +707,11 @@
           <t>Kompletní</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Žádost odeslána</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -728,6 +746,11 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>ne</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>připraveno, čeká na konektor</t>
         </is>
       </c>
     </row>
@@ -742,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -753,6 +776,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -794,6 +818,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Kompletní</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Žádost odeslána</t>
         </is>
       </c>
     </row>
@@ -848,7 +877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -859,6 +888,7 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -900,6 +930,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Kompletní</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Žádost odeslána</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cvičný projekt jde doopravdy spustit, lekce popisuje ten běh
Evidence se ve stahovaném projektu vezla už naplněná všemi pěti řádky.
Skill přitom zpracovává PDF, která řádek ještě nemají — takže první běh
neudělal nic, přestože lekce slibuje „stáhneš, pustíš, porovnáš". Teď
objednavky.xlsx veze jen hlavičky sloupců a běh ho naplní.

Sekce 3 popisovala živou schránku, kterou účastník při prvním spuštění
nemá. Nově popisuje ten běh, co se doopravdy stane: pět faktur ve vstup/,
čtyři kompletní, Elektro Dvořák bez čísla objednávky, text připravený a
neodeslaný, protokol — a druhé spuštění, které správně neudělá nic. Co
se změní po napojení schránky, je vedle v poznámce.

Přibývá diagram kontrola-flow: čtyři kroky a rozcestí podle počtu
chybějících údajů, protože tam se rozhoduje, jestli něco odejde ven.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cviceni/faktury-kontrola/data/objednavky.xlsx
+++ b/cviceni/faktury-kontrola/data/objednavky.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -489,46 +489,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-09-01_stavebniny-morava.pdf</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1. 9. 2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>FA-2026-0918</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>27182934</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OBJ-2026-0442</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>48250</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>22. 9. 2026</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -540,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -601,46 +561,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-09-02_naradi-profi.pdf</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2. 9. 2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>FA-2026-0919</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>45319876</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OBJ-2026-0447</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>12900</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>25. 9. 2026</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -652,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -713,47 +633,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-03_elektro-dvorak.pdf</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>3. 9. 2026</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2026/1044</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>61234567</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="n">
-        <v>7340</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>30. 9. 2026</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>ne</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>připraveno, čeká na konektor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -765,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -826,46 +705,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-09-04_vts-technik.pdf</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>4. 9. 2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>FA-2026-0921</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>28374651</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OBJ-2026-0451</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>33100</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>28. 9. 2026</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -877,7 +716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -938,46 +777,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-09-05_barvy-piekarova.pdf</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>5. 9. 2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>FA-2026-0922</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>49876123</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OBJ-9999-0001</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>5480</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1. 10. 2026</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Přebalený zip z upravené složky
Ze složky přišly tři změny; do veřejné verze se propsala jedna.

README měl špatný počet míst, kde se přepisuje adresa: sliboval deset,
skutečnost je sedmnáct, a rozpad po souborech taky nesouhlasil (rutina.md
osmkrát, ne dvakrát; zadani.md čtyřikrát). Ověřeno počítáním, teď to sedí.

Podpis v šabloně e-mailu se ve složce změnil z „Účtárna DEK" na jméno.
Ve veřejné verzi zůstává role — je to jediné místo šablony, kde by jinak
stálo jméno konkrétního člověka.

Běh z 2026-09-10 do zipu nešel. Jeho protokol nese čtyři skutečné adresy
včetně jména člověka u dodavatele a systémové adresy skladu, a popisuje
práci s živou schránkou, kterou cvičný projekt bez konektoru stejně
nezopakuje. Referenční výstupy zůstávají 09-08 a 09-09, jak na ně README
odkazuje.

Evidence je zase vyprázdněná a sešit z živého testu vyndaný, aby první běh
u účastníků měl co dělat.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cviceni/faktury-kontrola/data/objednavky.xlsx
+++ b/cviceni/faktury-kontrola/data/objednavky.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5115" yWindow="855" windowWidth="21600" windowHeight="11295" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Stavebniny Morava" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Barvy Piekarová" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -54,15 +54,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normální" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -424,7 +423,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
@@ -489,7 +488,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
@@ -554,7 +553,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
@@ -619,7 +618,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
@@ -684,7 +683,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>

</xml_diff>